<commit_message>
Giai đoạn 13.6: cập nhật detail design theo các bản sửa lỗi; hoàn thành GĐ 13
- Chụp lại ảnh và sinh lại 12 file detail design bị ảnh hưởng (Tổng thể, Đơn thuê, Chi tiết đơn, Tạo/Sửa đơn,
  Gia hạn, Phòng, Thêm/Sửa phòng, Bảng giá, Phụ thu, Thêm/Sửa nhân viên, Lịch làm, Cài đặt), thêm lịch sử bản 1.1.
- Tạo/Sửa đơn có thêm ảnh "phòng còn khách quá giờ chưa trả" và "lưu khi thiếu ô bắt buộc"; Cài đặt có mục
  Xem trước mẫu tin nhắn; bỏ các ghi chú "đã báo lại" về lỗi đã sửa.
- Đánh dấu xong GĐ 13 và các lỗi phát hiện khi làm tài liệu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/detail-design/06_DonThue.xlsx
+++ b/docs/detail-design/06_DonThue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="145">
   <si>
     <t>SWEET HOME · DETAIL DESIGN · ĐƠN THUÊ</t>
   </si>
@@ -137,6 +137,12 @@
     <t>Tạo mới.</t>
   </si>
   <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>Số trên tab "Tất cả" luôn là tổng đơn mọi trạng thái (trước đây lấy total của tab đang chọn).</t>
+  </si>
+  <si>
     <t>Ảnh 1. Danh sách đơn (tab Tất cả)</t>
   </si>
   <si>
@@ -203,7 +209,7 @@
     <t>Tất cả</t>
   </si>
   <si>
-    <t>Tất cả · Đã đặt · Đang ở · Quá giờ · Chờ xác nhận · Đã trả · Đã huỷ. Số đếm theo bộ lọc phòng + ô tìm kiếm hiện tại (không theo tab); riêng tab Tất cả hiện tổng kết quả của tab đang chọn (sheet 4). Đổi tab về trang 1.</t>
+    <t>Tất cả · Đã đặt · Đang ở · Quá giờ · Chờ xác nhận · Đã trả · Đã huỷ. Số đếm theo bộ lọc phòng + ô tìm kiếm hiện tại (không theo tab); tab Tất cả = tổng số của mọi trạng thái (sheet 4). Đổi tab về trang 1.</t>
   </si>
   <si>
     <t>Ô tìm kiếm</t>
@@ -416,7 +422,7 @@
     <t>Trang (từ 0) và 10 đơn/trang; backend giới hạn size tối đa 100.</t>
   </si>
   <si>
-    <t>Kết quả: items (OrderDto, sắp giờ nhận giảm dần), total (tổng số đơn khớp bộ lọc + tab), countByStatus (số đơn theo từng trạng thái, áp bộ lọc phòng + tìm kiếm, không áp tab). Số trên các tab trạng thái lấy từ countByStatus; số trên tab "Tất cả" lấy từ total — khi đang ở tab khác, số này bằng số đơn của tab đang chọn chứ không phải tổng mọi trạng thái (hành vi hiện tại, đã báo lại để xem xét sửa).</t>
+    <t>Kết quả: items (OrderDto, sắp giờ nhận giảm dần), total (tổng số đơn khớp bộ lọc + tab), countByStatus (số đơn theo từng trạng thái, áp bộ lọc phòng + tìm kiếm, không áp tab). Số trên các tab trạng thái lấy từ countByStatus; số trên tab "Tất cả" = tổng các giá trị countByStatus (allCount), không phụ thuộc tab đang chọn. total chỉ dùng tính số trang.</t>
   </si>
   <si>
     <t>3. Hành động</t>
@@ -603,7 +609,7 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="9658350" cy="7740094"/>
+    <xdr:ext cx="9658350" cy="7102911"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -639,7 +645,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9658350" cy="6036468"/>
@@ -678,7 +684,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>80</xdr:row>
+      <xdr:row>77</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9658350" cy="6036468"/>
@@ -1041,7 +1047,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AG21"/>
+  <dimension ref="B1:AG22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1772,8 +1778,50 @@
       <c r="AF21" s="3"/>
       <c r="AG21" s="3"/>
     </row>
+    <row r="22" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+      <c r="U22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+      <c r="Y22" s="3"/>
+      <c r="Z22" s="3"/>
+      <c r="AA22" s="3"/>
+      <c r="AB22" s="3"/>
+      <c r="AC22" s="3"/>
+      <c r="AD22" s="3"/>
+      <c r="AE22" s="3"/>
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="43">
     <mergeCell ref="B1:AG1"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="I2:AG2"/>
@@ -1813,6 +1861,10 @@
     <mergeCell ref="E21:H21"/>
     <mergeCell ref="I21:M21"/>
     <mergeCell ref="N21:AG21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="I22:M22"/>
+    <mergeCell ref="N22:AG22"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -1823,7 +1875,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AG80"/>
+  <dimension ref="B1:AG77"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1832,7 +1884,7 @@
   <sheetData>
     <row r="1" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
@@ -1866,83 +1918,83 @@
       <c r="AF1" s="4"/>
       <c r="AG1" s="4"/>
     </row>
-    <row r="45" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B45" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
-      <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
-      <c r="P45" s="4"/>
-      <c r="Q45" s="4"/>
-      <c r="R45" s="4"/>
-      <c r="S45" s="4"/>
-      <c r="T45" s="4"/>
-      <c r="U45" s="4"/>
-      <c r="V45" s="4"/>
-      <c r="W45" s="4"/>
-      <c r="X45" s="4"/>
-      <c r="Y45" s="4"/>
-      <c r="Z45" s="4"/>
-      <c r="AA45" s="4"/>
-      <c r="AB45" s="4"/>
-      <c r="AC45" s="4"/>
-      <c r="AD45" s="4"/>
-      <c r="AE45" s="4"/>
-      <c r="AF45" s="4"/>
-      <c r="AG45" s="4"/>
-    </row>
-    <row r="80" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B80" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C80" s="4"/>
-      <c r="D80" s="4"/>
-      <c r="E80" s="4"/>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
-      <c r="H80" s="4"/>
-      <c r="I80" s="4"/>
-      <c r="J80" s="4"/>
-      <c r="K80" s="4"/>
-      <c r="L80" s="4"/>
-      <c r="M80" s="4"/>
-      <c r="N80" s="4"/>
-      <c r="O80" s="4"/>
-      <c r="P80" s="4"/>
-      <c r="Q80" s="4"/>
-      <c r="R80" s="4"/>
-      <c r="S80" s="4"/>
-      <c r="T80" s="4"/>
-      <c r="U80" s="4"/>
-      <c r="V80" s="4"/>
-      <c r="W80" s="4"/>
-      <c r="X80" s="4"/>
-      <c r="Y80" s="4"/>
-      <c r="Z80" s="4"/>
-      <c r="AA80" s="4"/>
-      <c r="AB80" s="4"/>
-      <c r="AC80" s="4"/>
-      <c r="AD80" s="4"/>
-      <c r="AE80" s="4"/>
-      <c r="AF80" s="4"/>
-      <c r="AG80" s="4"/>
+    <row r="42" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B42" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
+      <c r="Q42" s="4"/>
+      <c r="R42" s="4"/>
+      <c r="S42" s="4"/>
+      <c r="T42" s="4"/>
+      <c r="U42" s="4"/>
+      <c r="V42" s="4"/>
+      <c r="W42" s="4"/>
+      <c r="X42" s="4"/>
+      <c r="Y42" s="4"/>
+      <c r="Z42" s="4"/>
+      <c r="AA42" s="4"/>
+      <c r="AB42" s="4"/>
+      <c r="AC42" s="4"/>
+      <c r="AD42" s="4"/>
+      <c r="AE42" s="4"/>
+      <c r="AF42" s="4"/>
+      <c r="AG42" s="4"/>
+    </row>
+    <row r="77" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B77" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="4"/>
+      <c r="H77" s="4"/>
+      <c r="I77" s="4"/>
+      <c r="J77" s="4"/>
+      <c r="K77" s="4"/>
+      <c r="L77" s="4"/>
+      <c r="M77" s="4"/>
+      <c r="N77" s="4"/>
+      <c r="O77" s="4"/>
+      <c r="P77" s="4"/>
+      <c r="Q77" s="4"/>
+      <c r="R77" s="4"/>
+      <c r="S77" s="4"/>
+      <c r="T77" s="4"/>
+      <c r="U77" s="4"/>
+      <c r="V77" s="4"/>
+      <c r="W77" s="4"/>
+      <c r="X77" s="4"/>
+      <c r="Y77" s="4"/>
+      <c r="Z77" s="4"/>
+      <c r="AA77" s="4"/>
+      <c r="AB77" s="4"/>
+      <c r="AC77" s="4"/>
+      <c r="AD77" s="4"/>
+      <c r="AE77" s="4"/>
+      <c r="AF77" s="4"/>
+      <c r="AG77" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B1:AG1"/>
-    <mergeCell ref="B45:AG45"/>
-    <mergeCell ref="B80:AG80"/>
+    <mergeCell ref="B42:AG42"/>
+    <mergeCell ref="B77:AG77"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <drawing r:id="rId1"/>
@@ -1963,7 +2015,7 @@
   <sheetData>
     <row r="1" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
@@ -1999,10 +2051,10 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -2013,22 +2065,22 @@
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="R2" s="5"/>
       <c r="S2" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="T2" s="5"/>
       <c r="U2" s="5"/>
@@ -2036,12 +2088,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Z2" s="5"/>
       <c r="AA2" s="5"/>
       <c r="AB2" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AC2" s="5"/>
       <c r="AD2" s="5"/>
@@ -2054,33 +2106,33 @@
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R3" s="3"/>
       <c r="S3" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
@@ -2088,12 +2140,12 @@
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
@@ -2106,33 +2158,33 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
@@ -2140,12 +2192,12 @@
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="Z4" s="3"/>
       <c r="AA4" s="3"/>
       <c r="AB4" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
@@ -2158,33 +2210,33 @@
         <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
@@ -2192,12 +2244,12 @@
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
       <c r="Y5" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Z5" s="3"/>
       <c r="AA5" s="3"/>
       <c r="AB5" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
@@ -2210,33 +2262,33 @@
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
@@ -2244,12 +2296,12 @@
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="Z6" s="3"/>
       <c r="AA6" s="3"/>
       <c r="AB6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
@@ -2262,33 +2314,33 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
@@ -2296,12 +2348,12 @@
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
       <c r="Y7" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z7" s="3"/>
       <c r="AA7" s="3"/>
       <c r="AB7" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AC7" s="3"/>
       <c r="AD7" s="3"/>
@@ -2314,33 +2366,33 @@
         <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
@@ -2348,12 +2400,12 @@
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
       <c r="Y8" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z8" s="3"/>
       <c r="AA8" s="3"/>
       <c r="AB8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
@@ -2366,33 +2418,33 @@
         <v>7</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
@@ -2400,12 +2452,12 @@
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z9" s="3"/>
       <c r="AA9" s="3"/>
       <c r="AB9" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AC9" s="3"/>
       <c r="AD9" s="3"/>
@@ -2418,33 +2470,33 @@
         <v>8</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P10" s="3"/>
       <c r="Q10" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R10" s="3"/>
       <c r="S10" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -2452,12 +2504,12 @@
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
       <c r="Y10" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z10" s="3"/>
       <c r="AA10" s="3"/>
       <c r="AB10" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AC10" s="3"/>
       <c r="AD10" s="3"/>
@@ -2470,33 +2522,33 @@
         <v>9</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="P11" s="3"/>
       <c r="Q11" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R11" s="3"/>
       <c r="S11" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
@@ -2504,12 +2556,12 @@
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
       <c r="Y11" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z11" s="3"/>
       <c r="AA11" s="3"/>
       <c r="AB11" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AC11" s="3"/>
       <c r="AD11" s="3"/>
@@ -2522,33 +2574,33 @@
         <v>10</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P12" s="3"/>
       <c r="Q12" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
@@ -2556,12 +2608,12 @@
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
       <c r="Y12" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z12" s="3"/>
       <c r="AA12" s="3"/>
       <c r="AB12" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AC12" s="3"/>
       <c r="AD12" s="3"/>
@@ -2574,33 +2626,33 @@
         <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P13" s="3"/>
       <c r="Q13" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R13" s="3"/>
       <c r="S13" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
@@ -2608,12 +2660,12 @@
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z13" s="3"/>
       <c r="AA13" s="3"/>
       <c r="AB13" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
@@ -2623,7 +2675,7 @@
     </row>
     <row r="15" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -2659,10 +2711,10 @@
     </row>
     <row r="16" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
@@ -2673,22 +2725,22 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
       <c r="J16" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P16" s="5"/>
       <c r="Q16" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="R16" s="5"/>
       <c r="S16" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="T16" s="5"/>
       <c r="U16" s="5"/>
@@ -2696,12 +2748,12 @@
       <c r="W16" s="5"/>
       <c r="X16" s="5"/>
       <c r="Y16" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Z16" s="5"/>
       <c r="AA16" s="5"/>
       <c r="AB16" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AC16" s="5"/>
       <c r="AD16" s="5"/>
@@ -2714,33 +2766,33 @@
         <v>12</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P17" s="3"/>
       <c r="Q17" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R17" s="3"/>
       <c r="S17" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
@@ -2748,12 +2800,12 @@
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
       <c r="Y17" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
       <c r="AB17" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AC17" s="3"/>
       <c r="AD17" s="3"/>
@@ -2766,33 +2818,33 @@
         <v>13</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P18" s="3"/>
       <c r="Q18" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R18" s="3"/>
       <c r="S18" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
@@ -2800,12 +2852,12 @@
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
       <c r="Y18" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z18" s="3"/>
       <c r="AA18" s="3"/>
       <c r="AB18" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="AC18" s="3"/>
       <c r="AD18" s="3"/>
@@ -2815,7 +2867,7 @@
     </row>
     <row r="20" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -2851,10 +2903,10 @@
     </row>
     <row r="21" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B21" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
@@ -2865,22 +2917,22 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
       <c r="N21" s="5"/>
       <c r="O21" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P21" s="5"/>
       <c r="Q21" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="R21" s="5"/>
       <c r="S21" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="T21" s="5"/>
       <c r="U21" s="5"/>
@@ -2888,12 +2940,12 @@
       <c r="W21" s="5"/>
       <c r="X21" s="5"/>
       <c r="Y21" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Z21" s="5"/>
       <c r="AA21" s="5"/>
       <c r="AB21" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AC21" s="5"/>
       <c r="AD21" s="5"/>
@@ -2906,33 +2958,33 @@
         <v>14</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
       <c r="J22" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
       <c r="O22" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P22" s="3"/>
       <c r="Q22" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R22" s="3"/>
       <c r="S22" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
@@ -2940,12 +2992,12 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
       <c r="Y22" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Z22" s="3"/>
       <c r="AA22" s="3"/>
       <c r="AB22" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="AC22" s="3"/>
       <c r="AD22" s="3"/>
@@ -3113,7 +3165,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3149,7 +3201,7 @@
     </row>
     <row r="2" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -3185,10 +3237,10 @@
     </row>
     <row r="3" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -3223,10 +3275,10 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
@@ -3261,7 +3313,7 @@
     </row>
     <row r="6" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -3297,14 +3349,14 @@
     </row>
     <row r="7" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -3335,14 +3387,14 @@
     </row>
     <row r="8" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -3373,14 +3425,14 @@
     </row>
     <row r="9" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -3411,14 +3463,14 @@
     </row>
     <row r="10" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -3449,14 +3501,14 @@
     </row>
     <row r="11" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -3487,7 +3539,7 @@
     </row>
     <row r="12" ht="43" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -3523,7 +3575,7 @@
     </row>
     <row r="14" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3559,7 +3611,7 @@
     </row>
     <row r="15" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
@@ -3568,7 +3620,7 @@
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
@@ -3597,7 +3649,7 @@
     </row>
     <row r="16" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -3606,7 +3658,7 @@
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
@@ -3635,7 +3687,7 @@
     </row>
     <row r="17" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -3644,7 +3696,7 @@
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
@@ -3673,7 +3725,7 @@
     </row>
     <row r="18" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -3682,7 +3734,7 @@
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
@@ -3711,7 +3763,7 @@
     </row>
     <row r="19" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -3720,7 +3772,7 @@
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
@@ -3749,7 +3801,7 @@
     </row>
     <row r="20" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>

</xml_diff>